<commit_message>
Fill HSK2 parts 2 (ID 551-600) with parts of speech
</commit_message>
<xml_diff>
--- a/HSK2_parts_of_speech_2(551-600).xlsx
+++ b/HSK2_parts_of_speech_2(551-600).xlsx
@@ -644,6 +644,11 @@
           <t>луг, лужайка</t>
         </is>
       </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>луг, лужайка</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -670,6 +675,16 @@
           <t>этаж, ярус</t>
         </is>
       </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>этаж, ярус</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>для этажей и слоёв (三层楼 — три этажа; 一层灰 — слой пыли)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -696,6 +711,11 @@
           <t>наводить справки</t>
         </is>
       </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>наводить справки, проверять; искать (查字典 — искать в словаре); осматривать (体检检查)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -722,6 +742,16 @@
           <t>почти</t>
         </is>
       </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>примерно одинаковые</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>почти, примерно (差不多 — почти одинаково)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -748,6 +778,21 @@
           <t>длинный</t>
         </is>
       </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>расти, удлиняться (长高了 — вырос)</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>длинный; длинный по росту (个子长 — высокого роста)</t>
+        </is>
+      </c>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t>многозначен: cháng «длинный» (形容词/动词 «расти» см. соответствующие столбцы); как существительное — старшинство (排行) в книжном стиле</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -774,6 +819,16 @@
           <t>часто встречающийся</t>
         </is>
       </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>часто встречающийся, обычный</t>
+        </is>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>常+见: выступает как прилагательное/часть устойчивого сочетания</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -800,6 +855,16 @@
           <t>часто используемый</t>
         </is>
       </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>часто используемый</t>
+        </is>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>常+用: используется перед существительным (常用词 — частотное слово)</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -826,6 +891,16 @@
           <t>площадь</t>
         </is>
       </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>площадка, поле (操场 — спортплощадка)</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>для событий, представлений, погоды: 一场电影 (фильм), 一场雨 (дождь), 一场球 (игра)</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -852,6 +927,11 @@
           <t>превышать, превосходить</t>
         </is>
       </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>превышать, превосходить (超过三十岁 — старше тридцати)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -878,6 +958,11 @@
           <t>супермаркет</t>
         </is>
       </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>супермаркет</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -904,6 +989,11 @@
           <t>транспортное средство</t>
         </is>
       </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>транспортные средства (собирательное, книжное)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -930,6 +1020,11 @@
           <t>звать, называть</t>
         </is>
       </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>называть, звать (自称 — называть себя); взвешивать (称体重)</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -956,6 +1051,21 @@
           <t>становиться, завершаться</t>
         </is>
       </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>становиться (成为); удаваться, завершаться (没做成 — не удалось); составить (成语 — фразеологизм)</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>для групп/команд (分成三组 — разбиться на три группы)</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>变成, в знач. «в качестве» (把他当成朋友 — считать его другом)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -982,6 +1092,11 @@
           <t>достижение</t>
         </is>
       </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>успеваемость, результат, оценка (成绩很好 — отличные результаты)</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1008,6 +1123,11 @@
           <t>стать (кем-либо, чем-либо)</t>
         </is>
       </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>стать, стать кем-то/чем-то (成为医生 — стать врачом)</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1034,6 +1154,11 @@
           <t>повторять заново</t>
         </is>
       </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>повторять, повторяться (重复一遍 — повторить ещё раз)</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1060,6 +1185,11 @@
           <t>заново</t>
         </is>
       </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>заново, снова (重新开始 — начать заново)</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1086,6 +1216,16 @@
           <t>отправляться; исходить из...</t>
         </is>
       </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>отправляться в путь (出发吧!); исходить из (从实际出发现实出发)</t>
+        </is>
+      </c>
+      <c r="X19" t="inlineStr">
+        <is>
+          <t>离合词: 出过一次国 — разъединяется</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1112,6 +1252,16 @@
           <t>выезжать за границу</t>
         </is>
       </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>выезжать за границу (出国学习 — учиться за границей)</t>
+        </is>
+      </c>
+      <c r="X20" t="inlineStr">
+        <is>
+          <t>离合词: 出了两次国</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1138,6 +1288,16 @@
           <t>экспорт</t>
         </is>
       </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>экспорт (出口商品 — экспортные товары); выход (安全出口 — аварийный выход)</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>экспортировать</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1164,6 +1324,16 @@
           <t>выходить из дома</t>
         </is>
       </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>выходить из дома (快出门了 — скоро выхожу)</t>
+        </is>
+      </c>
+      <c r="X22" t="inlineStr">
+        <is>
+          <t>离合词: 出了一趟门</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1190,6 +1360,21 @@
           <t>рождаться</t>
         </is>
       </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>рождение, дата рождения</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>рождаться (出生在北京 — родился в Пекине)</t>
+        </is>
+      </c>
+      <c r="X23" t="inlineStr">
+        <is>
+          <t>离合词: 他出生于1990年</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1216,6 +1401,11 @@
           <t>появляться</t>
         </is>
       </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>появляться, возникать (出现问题 — появилась проблема)</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1242,6 +1432,16 @@
           <t>выписываться из больницы</t>
         </is>
       </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>выписываться из больницы (出院回家 — выписаться домой)</t>
+        </is>
+      </c>
+      <c r="X25" t="inlineStr">
+        <is>
+          <t>离合词: 刚出过院</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1268,6 +1468,16 @@
           <t>арендовать</t>
         </is>
       </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>сдавать в аренду, арендовать (出租房屋 — сдавать жильё)</t>
+        </is>
+      </c>
+      <c r="W26" t="inlineStr">
+        <is>
+          <t>используется перед сущ.: 出租车 (такси), 出租房 (арендованное жильё)</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1294,6 +1504,11 @@
           <t>такси</t>
         </is>
       </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>такси</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1320,6 +1535,16 @@
           <t>лодка</t>
         </is>
       </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>лодка, судно (坐船 — плыть на корабле)</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>для больших судов: 一条船 (редко, чаще 艘)</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1346,6 +1571,11 @@
           <t>дуть</t>
         </is>
       </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>дуть (风吹 — ветер дует); хвастаться (吹牛 — врать/хвастаться)</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1372,6 +1602,11 @@
           <t>Праздник Весны, китайский Новый год</t>
         </is>
       </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>Праздник Весны, китайский Новый год (春节 — главный праздник)</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -1398,6 +1633,11 @@
           <t>весна</t>
         </is>
       </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>весна (春天来了 — весна пришла)</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -1424,6 +1664,11 @@
           <t>слово</t>
         </is>
       </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>слово (生词 — новое слово); стихи, лирика (宋词 — поэзия эпохи Сун)</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -1450,6 +1695,11 @@
           <t>словарь</t>
         </is>
       </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>словарь (查词典 — посмотреть в словаре)</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -1476,6 +1726,11 @@
           <t>слово, оборот речи</t>
         </is>
       </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>слова и выражения, лексика (词语积累 — накопление лексики)</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -1502,6 +1757,16 @@
           <t>с детства</t>
         </is>
       </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>с детства (从小长大 — вырос с детства)</t>
+        </is>
+      </c>
+      <c r="X35" t="inlineStr">
+        <is>
+          <t>предложно-именное сочетание 从+小, цельная наречная единица</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -1528,6 +1793,11 @@
           <t>обещать, дать согласие</t>
         </is>
       </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>обещать, согласиться (答应他 — пообещать ему; 我答应了 — я согласен)</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -1554,6 +1824,16 @@
           <t>работать</t>
         </is>
       </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>подрабатывать, работать (прост.) (去打工 — пойти подрабатывать)</t>
+        </is>
+      </c>
+      <c r="X37" t="inlineStr">
+        <is>
+          <t>离合词: 打了一年工</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -1580,6 +1860,16 @@
           <t>планировать</t>
         </is>
       </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>планы, намерения (有什么打算 — какие у вас планы?)</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>собиратьcя, планировать (打算去 — собираюсь поехать)</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -1606,6 +1896,16 @@
           <t>печатать</t>
         </is>
       </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>печатать (打印文件 — распечатать документ)</t>
+        </is>
+      </c>
+      <c r="X39" t="inlineStr">
+        <is>
+          <t>离合词: 打印过几次</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -1632,6 +1932,16 @@
           <t>большая часть</t>
         </is>
       </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>большая часть (大部分人都同意 — большинство согласно)</t>
+        </is>
+      </c>
+      <c r="W40" t="inlineStr">
+        <is>
+          <t>перед сущ.: 大部分时间 — большая часть времени</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -1658,6 +1968,16 @@
           <t>значительно, в больших размерах</t>
         </is>
       </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>значительно, в большой степени (大大改善 — значительно улучшилось)</t>
+        </is>
+      </c>
+      <c r="X41" t="inlineStr">
+        <is>
+          <t>наречие редупликации, употребляется только перед глаголами</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -1684,6 +2004,16 @@
           <t>большинство</t>
         </is>
       </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>большинство (大多数学生 — большинство студентов)</t>
+        </is>
+      </c>
+      <c r="W42" t="inlineStr">
+        <is>
+          <t>перед сущ.: 大多数人 — большинство людей</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -1710,6 +2040,16 @@
           <t>море</t>
         </is>
       </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>море (大海边 — морской берег)</t>
+        </is>
+      </c>
+      <c r="X43" t="inlineStr">
+        <is>
+          <t>поэтическое/общее обозначение моря; конкретные моря — 太平洋 и т.п.</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -1736,6 +2076,11 @@
           <t>все</t>
         </is>
       </c>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>все, все присутствующие (大家来吧 — приходите все); великие люди (книжн.)</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -1762,6 +2107,21 @@
           <t>многие; массовый</t>
         </is>
       </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>большое количество (需要大量 — нужно много)</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>массовый, объёмный (大量生产 — массовое производство)</t>
+        </is>
+      </c>
+      <c r="W45" t="inlineStr">
+        <is>
+          <t>перед сущ.: 大量资料 — масса материалов</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -1788,6 +2148,11 @@
           <t>ворота, главный вход</t>
         </is>
       </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>главные ворота, парадный вход (大门口的牌子 — табличка у ворот)</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -1814,6 +2179,16 @@
           <t>взрослый</t>
         </is>
       </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>взрослый человек (大人和小孩 — взрослые и дети)</t>
+        </is>
+      </c>
+      <c r="W47" t="inlineStr">
+        <is>
+          <t>перед сущ.: 大人说话 — взрослый разговор</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -1840,6 +2215,16 @@
           <t>громко, во весь голос</t>
         </is>
       </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>громкий голос (大声欢呼 — радостно восклицать)</t>
+        </is>
+      </c>
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t>громко, во весь голос (大声说 — говорить громко)</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -1866,6 +2251,16 @@
           <t>размер</t>
         </is>
       </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>размер, величина (大小合适 — подходит по размеру)</t>
+        </is>
+      </c>
+      <c r="X49" t="inlineStr">
+        <is>
+          <t>субстантивированное соединение прилагательных 大+小</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -1892,6 +2287,11 @@
           <t>пальто</t>
         </is>
       </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>пальто (冬大衣 — зимнее пальто)</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -1916,6 +2316,16 @@
       <c r="I51" t="inlineStr">
         <is>
           <t>природа</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>природа (大自然的规律 — законы природы)</t>
+        </is>
+      </c>
+      <c r="W51" t="inlineStr">
+        <is>
+          <t>перед сущ.: 大自然的风光 — природные красоты</t>
         </is>
       </c>
     </row>

</xml_diff>